<commit_message>
Apply validated category sweep and document vocab update process
- Backprop 189 changes from validated union table to canonical CSV
  and vocabulary.json: 141 category fixes, 36 POS corrections,
  10 tab reassignments, 2 secondary_tabs additions
- Add 58 anchor memberships to meaning_room.json (T1-T3 words
  gaining spatial homes in the meaning room)
- Fix vocab_sync.py diff to handle secondary_tabs list comparison
- Fix truncated ui_tab value for 'already' (Func → more)
- Add docs/vocabulary-update-guide.md: end-to-end documentation
  of the validation sweep, backprop, and sync pipeline
</commit_message>
<xml_diff>
--- a/data/vocabulary_union_table.xlsx
+++ b/data/vocabulary_union_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mpesavento/src/lief-amiga/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC57B237-C959-D446-AE3D-AC86DD1B6194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23D241D7-ECA0-CC4B-AEAC-73B2A37DBF76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="35120" yWindow="-11220" windowWidth="22320" windowHeight="19560" xr2:uid="{0BB74483-E000-414E-9A7C-48B773B8CC6A}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3917" uniqueCount="725">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3917" uniqueCount="724">
   <si>
     <t>symbol_id</t>
   </si>
@@ -2187,9 +2187,6 @@
   </si>
   <si>
     <t>cross-cutting: i_want_water</t>
-  </si>
-  <si>
-    <t>Func</t>
   </si>
   <si>
     <t>we_ll</t>
@@ -11062,7 +11059,7 @@
         <v>476</v>
       </c>
       <c r="F247" t="s">
-        <v>722</v>
+        <v>77</v>
       </c>
       <c r="H247" t="s">
         <v>18</v>
@@ -15535,7 +15532,7 @@
     </row>
     <row r="400" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A400" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B400" t="s">
         <v>652</v>
@@ -15564,7 +15561,7 @@
     </row>
     <row r="401" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A401" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="B401" t="s">
         <v>653</v>

</xml_diff>